<commit_message>
Actualziacion del INFORME ANS  ATC CHEC V2
</commit_message>
<xml_diff>
--- a/config/DIAS_CONTRACTUALES.xlsx
+++ b/config/DIAS_CONTRACTUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hector.gaviria\Desktop\Informe_ANS_ATC_CHEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25E142E-3665-4FBF-913C-E0F3E6DAFD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1750FA-CB29-4156-A324-D0A39BD07ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="3" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="184">
   <si>
     <t xml:space="preserve">MUNICIPIOS </t>
   </si>
@@ -532,15 +532,6 @@
     <t>VALOR</t>
   </si>
   <si>
-    <t>DIAS_MUNICIPIO_NO_CONFIGURADO</t>
-  </si>
-  <si>
-    <t>Días pactados para municipios que no aparecen en REGLAS_DE_NEGOCIO</t>
-  </si>
-  <si>
-    <t>UMBRAL_ALERTA_DIAS</t>
-  </si>
-  <si>
     <t>Cantidad de días restantes para clasificar un pedido como ALERTA</t>
   </si>
   <si>
@@ -644,6 +635,21 @@
   </si>
   <si>
     <t>ACTIVO</t>
+  </si>
+  <si>
+    <t>DIAS_INICIO_ALERTA</t>
+  </si>
+  <si>
+    <t>Una vez la fecha límite ya fue superada (días restantes negativos), el pedido se clasifica como VENCIDO.</t>
+  </si>
+  <si>
+    <t>Si aún le restan más de 2 días, el pedido se considera A TIEMPO.</t>
+  </si>
+  <si>
+    <t>DIAS_INICIO_ALERTA = 2 significa que un pedido pasa al estado ALERTA cuando le restan 2 días o o menos para vencer.</t>
+  </si>
+  <si>
+    <t>ESTADOS</t>
   </si>
 </sst>
 </file>
@@ -655,7 +661,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -686,8 +692,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -706,8 +727,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -809,13 +842,93 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -911,6 +1024,23 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -937,34 +1067,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1048,6 +1150,34 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1062,23 +1192,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A1:B32" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C7" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:C7" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="11">
+  <autoFilter ref="A1:C6" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1534,7 +1664,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B10" s="28">
         <v>7</v>
@@ -1542,7 +1672,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B11" s="28">
         <v>7</v>
@@ -1550,7 +1680,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B12" s="28">
         <v>7</v>
@@ -1558,7 +1688,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B13" s="28">
         <v>7</v>
@@ -1566,7 +1696,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B14" s="28">
         <v>7</v>
@@ -1574,7 +1704,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B15" s="28">
         <v>7</v>
@@ -1582,7 +1712,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B16" s="28">
         <v>7</v>
@@ -1590,7 +1720,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B17" s="28">
         <v>7</v>
@@ -1598,7 +1728,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B18" s="28">
         <v>7</v>
@@ -1606,7 +1736,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B19" s="28">
         <v>7</v>
@@ -1614,7 +1744,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B20" s="28">
         <v>7</v>
@@ -1622,7 +1752,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B21" s="28">
         <v>7</v>
@@ -1630,7 +1760,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B22" s="28">
         <v>7</v>
@@ -1638,7 +1768,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B23" s="28">
         <v>7</v>
@@ -1646,7 +1776,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B24" s="28">
         <v>7</v>
@@ -1654,7 +1784,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B25" s="28">
         <v>7</v>
@@ -1662,7 +1792,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B26" s="28">
         <v>7</v>
@@ -1670,7 +1800,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="31" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B27" s="28">
         <v>7</v>
@@ -1678,7 +1808,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="31" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B28" s="28">
         <v>7</v>
@@ -1686,7 +1816,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B29" s="28">
         <v>7</v>
@@ -1694,7 +1824,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="31" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B30" s="28">
         <v>7</v>
@@ -1702,7 +1832,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="31" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B31" s="28">
         <v>7</v>
@@ -1710,7 +1840,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B32" s="28">
         <v>7</v>
@@ -1729,7 +1859,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22D2DA52-4543-4DA0-B58A-301AB3B9677B}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="81" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
@@ -1750,21 +1880,21 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" s="17">
+        <v>2</v>
+      </c>
+      <c r="C2" s="30" t="s">
         <v>144</v>
-      </c>
-      <c r="B2" s="17">
-        <v>7</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>146</v>
-      </c>
-      <c r="B3" s="17">
-        <v>2</v>
       </c>
       <c r="C3" s="30" t="s">
         <v>147</v>
@@ -1775,46 +1905,64 @@
         <v>148</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="30" t="s">
         <v>149</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="30" t="s">
         <v>151</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>156</v>
-      </c>
+    </row>
+    <row r="11" spans="1:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="36" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="43" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="44"/>
+      <c r="C12" s="45"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="B13" s="37"/>
+      <c r="C13" s="38"/>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="39" t="s">
+        <v>180</v>
+      </c>
+      <c r="B14" s="40"/>
+      <c r="C14" s="41"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:C12"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1824,7 +1972,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4947552-E839-4268-808D-3A4D510046FA}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="14.42578125" customWidth="1"/>
@@ -1832,14 +1980,17 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B1" t="s">
         <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>181</v>
-      </c>
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="35"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualziacion del INFORME ANS  ATC CHEC V5
</commit_message>
<xml_diff>
--- a/config/DIAS_CONTRACTUALES.xlsx
+++ b/config/DIAS_CONTRACTUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hector.gaviria\Desktop\Informe_ANS_ATC_CHEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1750FA-CB29-4156-A324-D0A39BD07ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01061EE-E513-4FB8-8446-134885100C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId1"/>
@@ -1026,12 +1026,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1039,6 +1033,24 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1067,6 +1079,34 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1150,34 +1190,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1192,23 +1204,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="A1:B32" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:C6" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1939,29 +1951,31 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="45"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="39"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="38"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="42"/>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39" t="s">
+      <c r="A14" s="43" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="41"/>
+      <c r="B14" s="44"/>
+      <c r="C14" s="45"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Se actualiza el informe ANS ATC_CHEC
</commit_message>
<xml_diff>
--- a/config/DIAS_CONTRACTUALES.xlsx
+++ b/config/DIAS_CONTRACTUALES.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hector.gaviria\Desktop\Informe_ANS_ATC_CHEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01061EE-E513-4FB8-8446-134885100C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E68319BF-28E7-47A7-ACA8-A8063D6EF777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="4" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId1"/>
     <sheet name="REGLAS_DE_NEGOCIO" sheetId="4" r:id="rId2"/>
     <sheet name="PARAMETROS" sheetId="5" r:id="rId3"/>
     <sheet name="FESTIVOS_ADICIONALES" sheetId="6" r:id="rId4"/>
-    <sheet name="EJECUCION " sheetId="1" r:id="rId5"/>
-    <sheet name="MUNICIPIOS" sheetId="3" r:id="rId6"/>
+    <sheet name="REGLAS_PRIORIDAD" sheetId="7" r:id="rId5"/>
+    <sheet name="EJECUCION " sheetId="1" r:id="rId6"/>
+    <sheet name="MUNICIPIOS" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'EJECUCION '!$A$19:$K$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">MUNICIPIOS!$B$1:$C$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'EJECUCION '!$A$19:$K$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">MUNICIPIOS!$B$1:$C$22</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="190">
   <si>
     <t xml:space="preserve">MUNICIPIOS </t>
   </si>
@@ -650,6 +651,24 @@
   </si>
   <si>
     <t>ESTADOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">factibilidad </t>
+  </si>
+  <si>
+    <t>HV</t>
+  </si>
+  <si>
+    <t>PALABRA_CLAVE</t>
+  </si>
+  <si>
+    <t>DIAS</t>
+  </si>
+  <si>
+    <t>FACTIBILIDAD</t>
+  </si>
+  <si>
+    <t>INMEDIATO</t>
   </si>
 </sst>
 </file>
@@ -928,7 +947,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1026,6 +1045,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1038,7 +1061,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1059,7 +1082,37 @@
     <cellStyle name="Moneda" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1190,6 +1243,9 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1204,23 +1260,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12" totalsRowBorderDxfId="11">
   <autoFilter ref="A1:B32" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A1:C6" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0F28DC9A-38FC-4EFF-9FE3-EA8398510518}" name="Tabla4" displayName="Tabla4" ref="A1:C4" totalsRowShown="0" headerRowDxfId="15">
+  <autoFilter ref="A1:C4" xr:uid="{0F28DC9A-38FC-4EFF-9FE3-EA8398510518}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{305F09D3-70C3-4E78-A983-BA38BA26DC9E}" name="PALABRA_CLAVE"/>
+    <tableColumn id="3" xr3:uid="{1492C246-0DC4-4378-AFA1-B226A498D0C1}" name="TIPO"/>
+    <tableColumn id="2" xr3:uid="{8A43306C-FD6F-45EA-B9C1-3D23507319AE}" name="DIAS"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1860,7 +1928,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1951,25 +2019,25 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="39" t="s">
         <v>182</v>
       </c>
-      <c r="B12" s="38"/>
-      <c r="C12" s="39"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="41"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="40" t="s">
+      <c r="A13" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="B13" s="41"/>
-      <c r="C13" s="42"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="44"/>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="43" t="s">
+      <c r="A14" s="45" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="45"/>
+      <c r="B14" s="46"/>
+      <c r="C14" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2012,6 +2080,76 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA24B9E6-66B9-4106-A5B3-55D11F1E49FD}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="57.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:B2">
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4718A26-F49B-4A7D-B1B2-6AC7D2FF2CCE}">
   <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2786,12 +2924,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E49BB65A-5570-426E-93B8-21AC0C258021}">
   <dimension ref="B1:J22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="72.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.42578125" customWidth="1"/>
+    <col min="6" max="6" width="3.85546875" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
     <col min="9" max="9" width="38.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2994,6 +3135,12 @@
       <c r="D13">
         <v>15</v>
       </c>
+      <c r="I13" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="J13" s="38">
+        <v>4</v>
+      </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
@@ -3005,6 +3152,12 @@
       <c r="D14">
         <v>3</v>
       </c>
+      <c r="I14" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="J14" s="38">
+        <v>15</v>
+      </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
@@ -3016,6 +3169,12 @@
       <c r="D15">
         <v>4</v>
       </c>
+      <c r="I15" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="J15" s="38">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
@@ -3097,7 +3256,7 @@
   </sheetData>
   <autoFilter ref="B1:C22" xr:uid="{E49BB65A-5570-426E-93B8-21AC0C258021}"/>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Se actualzia los diseños del atc-chec
</commit_message>
<xml_diff>
--- a/config/DIAS_CONTRACTUALES.xlsx
+++ b/config/DIAS_CONTRACTUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hector.gaviria\Desktop\Informe_ANS_ATC_CHEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E68319BF-28E7-47A7-ACA8-A8063D6EF777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEB55F2-450D-4BE4-B20D-6FBEE73C5D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="4" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
+    <workbookView xWindow="-20610" yWindow="435" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="197">
   <si>
     <t xml:space="preserve">MUNICIPIOS </t>
   </si>
@@ -670,6 +670,27 @@
   <si>
     <t>INMEDIATO</t>
   </si>
+  <si>
+    <t>INMEDIATO: Servicio temporal urbano/Servicio temporal urbano</t>
+  </si>
+  <si>
+    <t>HV:Solicitud de conexión /Habilitación de Vivienda integral urbano</t>
+  </si>
+  <si>
+    <t>FACTIBILIDAD:Factibilidad del servicio/Cuenta nueva</t>
+  </si>
+  <si>
+    <t>COLORES</t>
+  </si>
+  <si>
+    <t>ALERTA</t>
+  </si>
+  <si>
+    <t>A TIEMPO</t>
+  </si>
+  <si>
+    <t>VENCIDO</t>
+  </si>
 </sst>
 </file>
 
@@ -680,7 +701,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -713,21 +734,27 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="16"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -748,18 +775,41 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF17A589"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -861,86 +911,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1044,45 +1014,35 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Moneda" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="17">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1134,32 +1094,17 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1244,7 +1189,32 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1260,30 +1230,30 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12" totalsRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="A1:B32" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="16">
   <autoFilter ref="A1:C6" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0F28DC9A-38FC-4EFF-9FE3-EA8398510518}" name="Tabla4" displayName="Tabla4" ref="A1:C4" totalsRowShown="0" headerRowDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0F28DC9A-38FC-4EFF-9FE3-EA8398510518}" name="Tabla4" displayName="Tabla4" ref="A1:C4" totalsRowShown="0" headerRowDxfId="6">
   <autoFilter ref="A1:C4" xr:uid="{0F28DC9A-38FC-4EFF-9FE3-EA8398510518}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{305F09D3-70C3-4E78-A983-BA38BA26DC9E}" name="PALABRA_CLAVE"/>
@@ -1928,7 +1898,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1939,15 +1909,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22D2DA52-4543-4DA0-B58A-301AB3B9677B}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="81" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="67" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
         <v>142</v>
       </c>
@@ -1958,7 +1929,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>179</v>
       </c>
@@ -1969,7 +1940,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="30" t="s">
         <v>145</v>
       </c>
@@ -1980,7 +1951,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="30" t="s">
         <v>148</v>
       </c>
@@ -1991,7 +1962,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
         <v>150</v>
       </c>
@@ -2002,7 +1973,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
         <v>152</v>
       </c>
@@ -2013,41 +1984,93 @@
         <v>153</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="36" t="s">
+    <row r="11" spans="1:4" ht="21" x14ac:dyDescent="0.35">
+      <c r="A11" s="41" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="38" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="42" t="s">
         <v>182</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="41"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="43" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="44"/>
-    </row>
-    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="45" t="s">
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="44" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="47"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="45" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="42" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="46" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="42" t="s">
+        <v>190</v>
+      </c>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="47" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="40" t="s">
+        <v>192</v>
+      </c>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="39" t="s">
+        <v>188</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="7">
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A15:C15"/>
   </mergeCells>
+  <conditionalFormatting sqref="A16">
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2133,14 +2156,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B2">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A3">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:B2">
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -3135,10 +3158,10 @@
       <c r="D13">
         <v>15</v>
       </c>
-      <c r="I13" s="37" t="s">
+      <c r="I13" s="36" t="s">
         <v>184</v>
       </c>
-      <c r="J13" s="38">
+      <c r="J13" s="37">
         <v>4</v>
       </c>
     </row>
@@ -3152,10 +3175,10 @@
       <c r="D14">
         <v>3</v>
       </c>
-      <c r="I14" s="38" t="s">
+      <c r="I14" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="J14" s="38">
+      <c r="J14" s="37">
         <v>15</v>
       </c>
     </row>
@@ -3169,10 +3192,10 @@
       <c r="D15">
         <v>4</v>
       </c>
-      <c r="I15" s="38" t="s">
+      <c r="I15" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="J15" s="38">
+      <c r="J15" s="37">
         <v>0</v>
       </c>
     </row>
@@ -3256,7 +3279,7 @@
   </sheetData>
   <autoFilter ref="B1:C22" xr:uid="{E49BB65A-5570-426E-93B8-21AC0C258021}"/>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Se actualzia el diseño de atc-chec
</commit_message>
<xml_diff>
--- a/config/DIAS_CONTRACTUALES.xlsx
+++ b/config/DIAS_CONTRACTUALES.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEB55F2-450D-4BE4-B20D-6FBEE73C5D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="435" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId1"/>
@@ -1022,20 +1022,20 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -1985,71 +1985,71 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="46" t="s">
         <v>183</v>
       </c>
-      <c r="B11" s="41"/>
-      <c r="C11" s="41"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
       <c r="D11" s="38" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="47" t="s">
         <v>182</v>
       </c>
-      <c r="B12" s="42"/>
-      <c r="C12" s="42"/>
-      <c r="D12" s="43" t="s">
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="40" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="47" t="s">
         <v>181</v>
       </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="44" t="s">
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="41" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="42" t="s">
+      <c r="A14" s="47" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="45" t="s">
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="42" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="42" t="s">
+      <c r="A15" s="47" t="s">
         <v>191</v>
       </c>
-      <c r="B15" s="42"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="46" t="s">
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="43" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="47" t="s">
         <v>190</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="47" t="s">
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="44" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="45" t="s">
         <v>192</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
       <c r="D17" s="39" t="s">
         <v>188</v>
       </c>

</xml_diff>

<commit_message>
Se actualizan el desarrollo ATC-CHEC
</commit_message>
<xml_diff>
--- a/config/DIAS_CONTRACTUALES.xlsx
+++ b/config/DIAS_CONTRACTUALES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hector.gaviria\Desktop\Informe_ANS_ATC_CHEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEB55F2-450D-4BE4-B20D-6FBEE73C5D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394F4798-5C0E-4EE4-8A3C-593B0DDFDF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="231">
   <si>
     <t xml:space="preserve">MUNICIPIOS </t>
   </si>
@@ -503,9 +503,6 @@
     <t>Municipio</t>
   </si>
   <si>
-    <t>Villa María</t>
-  </si>
-  <si>
     <t>Chinchina</t>
   </si>
   <si>
@@ -690,6 +687,111 @@
   </si>
   <si>
     <t>VENCIDO</t>
+  </si>
+  <si>
+    <t>Victoria</t>
+  </si>
+  <si>
+    <t>Pacora</t>
+  </si>
+  <si>
+    <t>Balboa</t>
+  </si>
+  <si>
+    <t>Santuario</t>
+  </si>
+  <si>
+    <t>Apia</t>
+  </si>
+  <si>
+    <t>Arauca</t>
+  </si>
+  <si>
+    <t>Arboleda</t>
+  </si>
+  <si>
+    <t>Arma</t>
+  </si>
+  <si>
+    <t>Belalcazar</t>
+  </si>
+  <si>
+    <t>Berlín</t>
+  </si>
+  <si>
+    <t>Bolivia</t>
+  </si>
+  <si>
+    <t>Buenavista</t>
+  </si>
+  <si>
+    <t>Castilla</t>
+  </si>
+  <si>
+    <t>Pereira</t>
+  </si>
+  <si>
+    <t>Florencia</t>
+  </si>
+  <si>
+    <t>Herveo</t>
+  </si>
+  <si>
+    <t>Irra</t>
+  </si>
+  <si>
+    <t>Isaza</t>
+  </si>
+  <si>
+    <t>Manzanares</t>
+  </si>
+  <si>
+    <t>Mariquita</t>
+  </si>
+  <si>
+    <t>Marquetalia</t>
+  </si>
+  <si>
+    <t>Marulanda</t>
+  </si>
+  <si>
+    <t>Montebonito</t>
+  </si>
+  <si>
+    <t>Pueblo Nuevo</t>
+  </si>
+  <si>
+    <t>Puerto Venus</t>
+  </si>
+  <si>
+    <t>Samaria</t>
+  </si>
+  <si>
+    <t>San Bartolomé</t>
+  </si>
+  <si>
+    <t>San Clemente</t>
+  </si>
+  <si>
+    <t>San Daniel</t>
+  </si>
+  <si>
+    <t>San Diego</t>
+  </si>
+  <si>
+    <t>San Félix</t>
+  </si>
+  <si>
+    <t>Santa Cecilia</t>
+  </si>
+  <si>
+    <t>Villa Claret</t>
+  </si>
+  <si>
+    <t>Villamaria</t>
+  </si>
+  <si>
+    <t>Tado</t>
   </si>
 </sst>
 </file>
@@ -701,7 +803,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -752,6 +854,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -917,7 +1025,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1009,9 +1117,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1027,6 +1132,12 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1105,6 +1216,34 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1188,34 +1327,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1230,23 +1341,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B32" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
-  <autoFilter ref="A1:B32" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B66" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+  <autoFilter ref="A1:B66" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="10">
   <autoFilter ref="A1:C6" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1634,7 +1745,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A5A6C8-8AB2-430A-814A-CCA4A30EF7E2}">
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
@@ -1645,7 +1756,7 @@
         <v>133</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1657,8 +1768,8 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
-        <v>134</v>
+      <c r="A3" s="44" t="s">
+        <v>229</v>
       </c>
       <c r="B3" s="28">
         <v>3</v>
@@ -1666,7 +1777,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B4" s="28">
         <v>3</v>
@@ -1674,7 +1785,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B5" s="28">
         <v>3</v>
@@ -1682,7 +1793,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B6" s="28">
         <v>3</v>
@@ -1690,7 +1801,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B7" s="28">
         <v>3</v>
@@ -1698,7 +1809,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B8" s="28">
         <v>3</v>
@@ -1706,15 +1817,15 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="32" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" s="34">
+        <v>139</v>
+      </c>
+      <c r="B9" s="33">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B10" s="28">
         <v>7</v>
@@ -1722,7 +1833,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B11" s="28">
         <v>7</v>
@@ -1730,7 +1841,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B12" s="28">
         <v>7</v>
@@ -1738,7 +1849,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B13" s="28">
         <v>7</v>
@@ -1746,7 +1857,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B14" s="28">
         <v>7</v>
@@ -1754,7 +1865,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B15" s="28">
         <v>7</v>
@@ -1762,7 +1873,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B16" s="28">
         <v>7</v>
@@ -1770,7 +1881,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B17" s="28">
         <v>7</v>
@@ -1778,7 +1889,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B18" s="28">
         <v>7</v>
@@ -1786,7 +1897,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B19" s="28">
         <v>7</v>
@@ -1794,7 +1905,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B20" s="28">
         <v>7</v>
@@ -1802,7 +1913,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B21" s="28">
         <v>7</v>
@@ -1810,7 +1921,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B22" s="28">
         <v>7</v>
@@ -1818,7 +1929,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B23" s="28">
         <v>7</v>
@@ -1826,7 +1937,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B24" s="28">
         <v>7</v>
@@ -1834,7 +1945,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B25" s="28">
         <v>7</v>
@@ -1842,7 +1953,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B26" s="28">
         <v>7</v>
@@ -1850,7 +1961,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="31" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B27" s="28">
         <v>7</v>
@@ -1858,7 +1969,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="31" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B28" s="28">
         <v>7</v>
@@ -1866,7 +1977,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B29" s="28">
         <v>7</v>
@@ -1874,7 +1985,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="31" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B30" s="28">
         <v>7</v>
@@ -1882,7 +1993,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="31" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B31" s="28">
         <v>7</v>
@@ -1890,9 +2001,281 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B32" s="28">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="B33" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="32" t="s">
+        <v>197</v>
+      </c>
+      <c r="B34" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="B35" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="B36" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="32" t="s">
+        <v>200</v>
+      </c>
+      <c r="B37" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="44" t="s">
+        <v>201</v>
+      </c>
+      <c r="B38" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B39" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="B40" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="44" t="s">
+        <v>204</v>
+      </c>
+      <c r="B41" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="44" t="s">
+        <v>205</v>
+      </c>
+      <c r="B42" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="44" t="s">
+        <v>206</v>
+      </c>
+      <c r="B43" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="B44" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="B45" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="44" t="s">
+        <v>209</v>
+      </c>
+      <c r="B46" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="B47" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="44" t="s">
+        <v>211</v>
+      </c>
+      <c r="B48" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="44" t="s">
+        <v>212</v>
+      </c>
+      <c r="B49" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="44" t="s">
+        <v>213</v>
+      </c>
+      <c r="B50" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="44" t="s">
+        <v>214</v>
+      </c>
+      <c r="B51" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="B52" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="B53" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="44" t="s">
+        <v>217</v>
+      </c>
+      <c r="B54" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="44" t="s">
+        <v>218</v>
+      </c>
+      <c r="B55" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="B56" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="44" t="s">
+        <v>220</v>
+      </c>
+      <c r="B57" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="44" t="s">
+        <v>221</v>
+      </c>
+      <c r="B58" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="44" t="s">
+        <v>222</v>
+      </c>
+      <c r="B59" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="44" t="s">
+        <v>223</v>
+      </c>
+      <c r="B60" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="44" t="s">
+        <v>224</v>
+      </c>
+      <c r="B61" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="44" t="s">
+        <v>225</v>
+      </c>
+      <c r="B62" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="44" t="s">
+        <v>226</v>
+      </c>
+      <c r="B63" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="44" t="s">
+        <v>227</v>
+      </c>
+      <c r="B64" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="44" t="s">
+        <v>228</v>
+      </c>
+      <c r="B65" s="33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="45" t="s">
+        <v>230</v>
+      </c>
+      <c r="B66" s="33">
         <v>7</v>
       </c>
     </row>
@@ -1920,10 +2303,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" s="29" t="s">
         <v>142</v>
-      </c>
-      <c r="B1" s="29" t="s">
-        <v>143</v>
       </c>
       <c r="C1" s="29" t="s">
         <v>23</v>
@@ -1931,127 +2314,127 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B2" s="17">
         <v>2</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="C3" s="30" t="s">
         <v>146</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C4" s="30" t="s">
         <v>148</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C5" s="30" t="s">
         <v>150</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>152</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>153</v>
-      </c>
     </row>
     <row r="11" spans="1:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="A11" s="46" t="s">
-        <v>183</v>
-      </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="38" t="s">
+      <c r="A11" s="47" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="37" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="48" t="s">
+        <v>181</v>
+      </c>
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="39" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="40" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="48" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" s="48"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="40" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="47" t="s">
-        <v>181</v>
-      </c>
-      <c r="B13" s="47"/>
-      <c r="C13" s="47"/>
-      <c r="D13" s="41" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="48" t="s">
+        <v>179</v>
+      </c>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="41" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="47" t="s">
-        <v>180</v>
-      </c>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="42" t="s">
-        <v>196</v>
-      </c>
-    </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="47" t="s">
+      <c r="A15" s="48" t="s">
+        <v>190</v>
+      </c>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="42" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="48" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="43" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="46" t="s">
         <v>191</v>
       </c>
-      <c r="B15" s="47"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="43" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="47" t="s">
-        <v>190</v>
-      </c>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="44" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="45" t="s">
-        <v>192</v>
-      </c>
-      <c r="B17" s="45"/>
-      <c r="C17" s="45"/>
-      <c r="D17" s="39" t="s">
-        <v>188</v>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="38" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2085,17 +2468,17 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B1" t="s">
         <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="35"/>
+      <c r="A2" s="34"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2113,13 +2496,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>17</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2127,7 +2510,7 @@
         <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -2138,7 +2521,7 @@
         <v>97</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C3">
         <v>15</v>
@@ -2149,7 +2532,7 @@
         <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C4">
         <v>4</v>
@@ -3158,10 +3541,10 @@
       <c r="D13">
         <v>15</v>
       </c>
-      <c r="I13" s="36" t="s">
-        <v>184</v>
-      </c>
-      <c r="J13" s="37">
+      <c r="I13" s="35" t="s">
+        <v>183</v>
+      </c>
+      <c r="J13" s="36">
         <v>4</v>
       </c>
     </row>
@@ -3175,10 +3558,10 @@
       <c r="D14">
         <v>3</v>
       </c>
-      <c r="I14" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="J14" s="37">
+      <c r="I14" s="36" t="s">
+        <v>184</v>
+      </c>
+      <c r="J14" s="36">
         <v>15</v>
       </c>
     </row>
@@ -3192,10 +3575,10 @@
       <c r="D15">
         <v>4</v>
       </c>
-      <c r="I15" s="37" t="s">
+      <c r="I15" s="36" t="s">
         <v>112</v>
       </c>
-      <c r="J15" s="37">
+      <c r="J15" s="36">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Parametrizar porcentaje de alerta ANS desde Excel
</commit_message>
<xml_diff>
--- a/config/DIAS_CONTRACTUALES.xlsx
+++ b/config/DIAS_CONTRACTUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hector.gaviria\Desktop\Informe_ANS_ATC_CHEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394F4798-5C0E-4EE4-8A3C-593B0DDFDF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D87F4E-70FB-4C9B-87F4-20140545FAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{2B542373-C365-41B5-A008-86F351A2B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId1"/>
@@ -530,9 +530,6 @@
     <t>VALOR</t>
   </si>
   <si>
-    <t>Cantidad de días restantes para clasificar un pedido como ALERTA</t>
-  </si>
-  <si>
     <t>EXCLUIR_SABADOS</t>
   </si>
   <si>
@@ -635,9 +632,6 @@
     <t>ACTIVO</t>
   </si>
   <si>
-    <t>DIAS_INICIO_ALERTA</t>
-  </si>
-  <si>
     <t>Una vez la fecha límite ya fue superada (días restantes negativos), el pedido se clasifica como VENCIDO.</t>
   </si>
   <si>
@@ -792,6 +786,12 @@
   </si>
   <si>
     <t>Tado</t>
+  </si>
+  <si>
+    <t>Porcentaje de días pactados para iniciar ALERTA</t>
+  </si>
+  <si>
+    <t>PORCENTAJE_INICIO_ALERTA</t>
   </si>
 </sst>
 </file>
@@ -1025,7 +1025,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1138,6 +1138,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1216,34 +1219,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1327,6 +1302,34 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1341,23 +1344,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B66" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}" name="Tabla2" displayName="Tabla2" ref="A1:B66" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="A1:B66" xr:uid="{DA7B9D9A-88A5-44AC-802A-CAAD236BFD48}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{C52FFFBA-0A3E-417F-AB87-E59567CB54D7}" name="Municipio" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{EBA87F11-6FBB-4F69-8D4B-0EABCF0F514A}" name="Dias" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}" name="Tabla3" displayName="Tabla3" ref="A1:C6" totalsRowShown="0" headerRowDxfId="16">
   <autoFilter ref="A1:C6" xr:uid="{23689B5E-A21A-438B-8158-1CF17B13D7E1}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{29E4BD0E-FD41-4EDE-8CFD-80F64E4908C0}" name="PARAMETRO" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{F23D1401-D9CF-4801-A8F9-1E1CDF2B05C7}" name="VALOR" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{4504E27A-BAA8-42B9-8B4B-377DB8A103D8}" name="DESCRIPCION" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1769,7 +1772,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="44" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B3" s="28">
         <v>3</v>
@@ -1825,7 +1828,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B10" s="28">
         <v>7</v>
@@ -1833,7 +1836,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B11" s="28">
         <v>7</v>
@@ -1841,7 +1844,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B12" s="28">
         <v>7</v>
@@ -1849,7 +1852,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B13" s="28">
         <v>7</v>
@@ -1857,7 +1860,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B14" s="28">
         <v>7</v>
@@ -1865,7 +1868,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B15" s="28">
         <v>7</v>
@@ -1873,7 +1876,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B16" s="28">
         <v>7</v>
@@ -1881,7 +1884,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B17" s="28">
         <v>7</v>
@@ -1889,7 +1892,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B18" s="28">
         <v>7</v>
@@ -1897,7 +1900,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B19" s="28">
         <v>7</v>
@@ -1905,7 +1908,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B20" s="28">
         <v>7</v>
@@ -1913,7 +1916,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B21" s="28">
         <v>7</v>
@@ -1921,7 +1924,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B22" s="28">
         <v>7</v>
@@ -1929,7 +1932,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B23" s="28">
         <v>7</v>
@@ -1937,7 +1940,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B24" s="28">
         <v>7</v>
@@ -1945,7 +1948,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B25" s="28">
         <v>7</v>
@@ -1953,7 +1956,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B26" s="28">
         <v>7</v>
@@ -1961,7 +1964,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="31" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B27" s="28">
         <v>7</v>
@@ -1969,7 +1972,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="31" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B28" s="28">
         <v>7</v>
@@ -1977,7 +1980,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B29" s="28">
         <v>7</v>
@@ -1985,7 +1988,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="31" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B30" s="28">
         <v>7</v>
@@ -1993,7 +1996,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="31" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B31" s="28">
         <v>7</v>
@@ -2001,7 +2004,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B32" s="28">
         <v>7</v>
@@ -2009,7 +2012,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="32" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B33" s="33">
         <v>7</v>
@@ -2017,7 +2020,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="32" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B34" s="33">
         <v>7</v>
@@ -2025,7 +2028,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="32" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B35" s="33">
         <v>7</v>
@@ -2033,7 +2036,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="32" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B36" s="33">
         <v>7</v>
@@ -2041,7 +2044,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="32" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B37" s="33">
         <v>7</v>
@@ -2049,7 +2052,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="44" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B38" s="33">
         <v>7</v>
@@ -2057,7 +2060,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="44" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B39" s="33">
         <v>7</v>
@@ -2065,7 +2068,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="44" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B40" s="33">
         <v>7</v>
@@ -2073,7 +2076,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="44" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B41" s="33">
         <v>7</v>
@@ -2081,7 +2084,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="44" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B42" s="33">
         <v>7</v>
@@ -2089,7 +2092,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="44" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B43" s="33">
         <v>7</v>
@@ -2097,7 +2100,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="44" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B44" s="33">
         <v>7</v>
@@ -2105,7 +2108,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="44" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B45" s="33">
         <v>7</v>
@@ -2113,7 +2116,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="44" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B46" s="33">
         <v>7</v>
@@ -2121,7 +2124,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="44" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B47" s="33">
         <v>7</v>
@@ -2129,7 +2132,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="44" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B48" s="33">
         <v>7</v>
@@ -2137,7 +2140,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="44" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B49" s="33">
         <v>7</v>
@@ -2145,7 +2148,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="44" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B50" s="33">
         <v>7</v>
@@ -2153,7 +2156,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="44" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B51" s="33">
         <v>7</v>
@@ -2161,7 +2164,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="44" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B52" s="33">
         <v>7</v>
@@ -2169,7 +2172,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="44" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B53" s="33">
         <v>7</v>
@@ -2177,7 +2180,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="44" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B54" s="33">
         <v>7</v>
@@ -2185,7 +2188,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="44" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B55" s="33">
         <v>7</v>
@@ -2193,7 +2196,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="44" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B56" s="33">
         <v>7</v>
@@ -2201,7 +2204,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="44" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B57" s="33">
         <v>7</v>
@@ -2209,7 +2212,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="44" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B58" s="33">
         <v>7</v>
@@ -2217,7 +2220,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="44" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B59" s="33">
         <v>7</v>
@@ -2225,7 +2228,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="44" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B60" s="33">
         <v>7</v>
@@ -2233,7 +2236,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="44" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B61" s="33">
         <v>7</v>
@@ -2241,7 +2244,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="44" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B62" s="33">
         <v>7</v>
@@ -2249,7 +2252,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="44" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B63" s="33">
         <v>7</v>
@@ -2257,7 +2260,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="44" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B64" s="33">
         <v>7</v>
@@ -2265,7 +2268,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="44" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B65" s="33">
         <v>7</v>
@@ -2273,7 +2276,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="45" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B66" s="33">
         <v>7</v>
@@ -2314,127 +2317,127 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="B2" s="17">
-        <v>2</v>
+        <v>230</v>
+      </c>
+      <c r="B2" s="46">
+        <v>0.33</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>143</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="C3" s="30" t="s">
         <v>145</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="30" t="s">
         <v>147</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="30" t="s">
         <v>149</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>152</v>
-      </c>
     </row>
     <row r="11" spans="1:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="A11" s="47" t="s">
+      <c r="A11" s="48" t="s">
+        <v>180</v>
+      </c>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="37" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="49" t="s">
+        <v>179</v>
+      </c>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="39" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="49" t="s">
+        <v>178</v>
+      </c>
+      <c r="B13" s="49"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="40" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="49" t="s">
+        <v>177</v>
+      </c>
+      <c r="B14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="41" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="49" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" s="49"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="42" t="s">
         <v>182</v>
       </c>
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="37" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="48" t="s">
-        <v>181</v>
-      </c>
-      <c r="B12" s="48"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="39" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="48" t="s">
-        <v>180</v>
-      </c>
-      <c r="B13" s="48"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="40" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="B14" s="48"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="41" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="48" t="s">
-        <v>190</v>
-      </c>
-      <c r="B15" s="48"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="42" t="s">
-        <v>184</v>
-      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="48" t="s">
+      <c r="A16" s="49" t="s">
+        <v>187</v>
+      </c>
+      <c r="B16" s="49"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="43" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="47" t="s">
         <v>189</v>
       </c>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="43" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="46" t="s">
-        <v>191</v>
-      </c>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
       <c r="D17" s="38" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2468,13 +2471,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B1" t="s">
         <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2496,13 +2499,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>17</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2510,7 +2513,7 @@
         <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -2521,7 +2524,7 @@
         <v>97</v>
       </c>
       <c r="B3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C3">
         <v>15</v>
@@ -2532,7 +2535,7 @@
         <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C4">
         <v>4</v>
@@ -3542,7 +3545,7 @@
         <v>15</v>
       </c>
       <c r="I13" s="35" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="J13" s="36">
         <v>4</v>
@@ -3559,7 +3562,7 @@
         <v>3</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="J14" s="36">
         <v>15</v>

</xml_diff>